<commit_message>
add find files, fix bugs, change default GUI construction
</commit_message>
<xml_diff>
--- a/тесты/проверка зон/фк/Зоны.xlsx
+++ b/тесты/проверка зон/фк/Зоны.xlsx
@@ -87,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -102,9 +102,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="2" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -478,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -535,99 +532,29 @@
           <t>LVDS</t>
         </is>
       </c>
-      <c r="G2" s="6" t="inlineStr">
-        <is>
-          <t>1039.304-1187.776</t>
-        </is>
-      </c>
-      <c r="H2" s="6" t="inlineStr">
-        <is>
-          <t>1039.304-1187.776</t>
-        </is>
-      </c>
-      <c r="I2" s="6" t="inlineStr">
-        <is>
-          <t>1039.304-1187.776</t>
-        </is>
-      </c>
-      <c r="J2" s="6" t="inlineStr">
-        <is>
-          <t>148.472-296.944</t>
-        </is>
-      </c>
-      <c r="K2" s="6" t="inlineStr">
-        <is>
-          <t>296.944-445.416</t>
-        </is>
-      </c>
-      <c r="L2" s="6" t="inlineStr">
-        <is>
-          <t>445.416-593.888</t>
-        </is>
-      </c>
-      <c r="M2" s="6" t="inlineStr">
-        <is>
-          <t>593.888-742.36</t>
-        </is>
-      </c>
-      <c r="N2" s="6" t="inlineStr">
-        <is>
-          <t>742.36-890.832</t>
-        </is>
-      </c>
-      <c r="O2" s="6" t="inlineStr">
-        <is>
-          <t>890.832-1039.304</t>
-        </is>
-      </c>
-      <c r="P2" s="6" t="inlineStr">
-        <is>
-          <t>890.832-1039.304</t>
-        </is>
-      </c>
-      <c r="Q2" s="6" t="inlineStr">
-        <is>
-          <t>890.832-1039.304</t>
-        </is>
-      </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="G2" s="5" t="inlineStr">
+        <is>
+          <t>SATA</t>
+        </is>
+      </c>
+      <c r="H2" s="5" t="inlineStr">
+        <is>
+          <t>блок электроники</t>
+        </is>
+      </c>
+      <c r="I2" s="5" t="inlineStr">
         <is>
           <t>USB</t>
         </is>
       </c>
-      <c r="S2" s="6" t="inlineStr">
-        <is>
-          <t>480-960</t>
-        </is>
-      </c>
-      <c r="T2" s="6" t="inlineStr">
-        <is>
-          <t>480-960</t>
-        </is>
-      </c>
-      <c r="U2" s="6" t="inlineStr">
-        <is>
-          <t>480-960</t>
-        </is>
-      </c>
-      <c r="V2" s="6" t="inlineStr">
-        <is>
-          <t>960-1440</t>
-        </is>
-      </c>
-      <c r="W2" s="5" t="inlineStr">
-        <is>
-          <t>SATA</t>
-        </is>
-      </c>
-      <c r="X2" s="6" t="inlineStr">
-        <is>
-          <t>0.009-6000</t>
+      <c r="J2" s="5" t="inlineStr">
+        <is>
+          <t>100 Мбит/с "витая пара"</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="7" t="n">
+      <c r="A3" s="6" t="n">
         <v>3.14</v>
       </c>
       <c r="B3" s="3" t="n">
@@ -636,7 +563,7 @@
       <c r="C3" s="3" t="n">
         <v>42</v>
       </c>
-      <c r="D3" s="8" t="n">
+      <c r="D3" s="7" t="n">
         <v>19</v>
       </c>
       <c r="E3" s="4" t="n">
@@ -647,19 +574,14 @@
           <t>LVDS</t>
         </is>
       </c>
-      <c r="G3" s="6" t="inlineStr">
-        <is>
-          <t>1039.304-1187.776</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
-        <is>
-          <t>1039.304-1187.776</t>
-        </is>
-      </c>
-      <c r="I3" s="6" t="inlineStr">
-        <is>
-          <t>148.472-296.944</t>
+      <c r="G3" s="5" t="inlineStr">
+        <is>
+          <t>SATA</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="inlineStr">
+        <is>
+          <t>100 Мбит/с "витая пара"</t>
         </is>
       </c>
     </row>
@@ -667,13 +589,13 @@
       <c r="A4" s="2" t="n">
         <v>3.3</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="7" t="n">
         <v>37</v>
       </c>
-      <c r="C4" s="8" t="n">
+      <c r="C4" s="7" t="n">
         <v>19</v>
       </c>
-      <c r="D4" s="8" t="n">
+      <c r="D4" s="7" t="n">
         <v>9</v>
       </c>
       <c r="E4" s="4" t="n">
@@ -684,54 +606,14 @@
           <t>LVDS</t>
         </is>
       </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>1039.304-1187.776</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>148.472-296.944</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>296.944-445.416</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>445.416-593.888</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>593.888-742.36</t>
-        </is>
-      </c>
-      <c r="L4" s="6" t="inlineStr">
-        <is>
-          <t>742.36-890.832</t>
-        </is>
-      </c>
-      <c r="M4" s="6" t="inlineStr">
-        <is>
-          <t>890.832-1039.304</t>
-        </is>
-      </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>SATA</t>
         </is>
       </c>
-      <c r="O4" s="6" t="inlineStr">
-        <is>
-          <t>0.009-1500</t>
-        </is>
-      </c>
-      <c r="P4" s="6" t="inlineStr">
-        <is>
-          <t>0.009-6000</t>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>USB</t>
         </is>
       </c>
     </row>

</xml_diff>